<commit_message>
Add unused-parameter pipeline rules, May EI batch, and credential gitignore patterns.
Detect unused params from code and output fields; tag section 04 with Not in use, exclude from 05/06, and verify in pipeline. Archive prior inputs under input/old, add bootstrap scripts and generated Explanation docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/input/old/Structure_SKN_S_SW_01_20_USER_STATE.xlsx
+++ b/input/old/Structure_SKN_S_SW_01_20_USER_STATE.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Structure" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,31 +413,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Structure Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Field Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Component Type</t>
         </is>
@@ -468,17 +456,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Account ID</t>
+          <t>ACCNT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>XUACCNT</t>
+          <t>ACCNT</t>
         </is>
       </c>
     </row>
@@ -495,17 +483,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Creator of the User Master Record</t>
+          <t>ANAME</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>XUANAME</t>
+          <t>ANAME</t>
         </is>
       </c>
     </row>
@@ -517,22 +505,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BCDA1</t>
+          <t>BACKDAYS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Date of Last Password Change</t>
+          <t>BACKDAYS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>DATS(8)</t>
+          <t>INT4(10)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>XUBCDAT</t>
+          <t>BACKDAYS</t>
         </is>
       </c>
     </row>
@@ -549,17 +537,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>User Name in User Master Record</t>
+          <t>BNAME</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>XUBNAME</t>
+          <t>BNAME</t>
         </is>
       </c>
     </row>
@@ -576,17 +564,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>User group in user master maintenance</t>
+          <t>CLASS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>XUCLASS</t>
+          <t>CLASS</t>
         </is>
       </c>
     </row>
@@ -598,22 +586,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CODV1</t>
+          <t>DATE_REF_FLD</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Code Version of Password Hash Algorithm (Old Systems)</t>
+          <t>DATE_REF_FLD</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CHAR(1)</t>
+          <t>CHAR(30)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>XUCODEVERS</t>
+          <t>NAME_FELD</t>
         </is>
       </c>
     </row>
@@ -625,22 +613,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CODVN</t>
+          <t>DATUM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Code Version of Password Hash Algorithm (New Systems)</t>
+          <t>DATUM</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CHAR(1)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>XUCODEVER2</t>
+          <t>DATUM</t>
         </is>
       </c>
     </row>
@@ -657,7 +645,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SW: Duration In Time Units (defined separatly)</t>
+          <t>DURATION</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -667,7 +655,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>/SKN/E_SW_DURATION</t>
+          <t>DURATION</t>
         </is>
       </c>
     </row>
@@ -684,7 +672,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SW: Duration Unit</t>
+          <t>DURATION_UNIT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -694,7 +682,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>/SKN/E_SW_DURATION_UNIT</t>
+          <t>DURATION_UNIT</t>
         </is>
       </c>
     </row>
@@ -711,17 +699,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Creation Date of the User Master Record</t>
+          <t>ERDAT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DATS(8)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>XUERDAT</t>
+          <t>ERDAT</t>
         </is>
       </c>
     </row>
@@ -733,22 +721,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GLTGB</t>
+          <t>LANGU</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>User valid to</t>
+          <t>LANGU</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DATS(8)</t>
+          <t>CHAR(1)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>XUGLTGB</t>
+          <t>LANGU</t>
         </is>
       </c>
     </row>
@@ -760,22 +748,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GLTGV</t>
+          <t>LOCNT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>User valid from</t>
+          <t>LOCNT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DATS(8)</t>
+          <t>INT4(10)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>XUGLTGV</t>
+          <t>LOCNT</t>
         </is>
       </c>
     </row>
@@ -787,22 +775,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>INIT_PWD_ICON</t>
+          <t>MANAGE_IN_UTC</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SW: State Icon</t>
+          <t>MANAGE_IN_UTC</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CHAR(4)</t>
+          <t>CHAR(1)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/SKN/E_SW_STATE_ICON</t>
+          <t>MANAGE_IN_UTC</t>
         </is>
       </c>
     </row>
@@ -814,22 +802,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>LOCK_ICON</t>
+          <t>MODBE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SW: State Icon</t>
+          <t>MODBE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>CHAR(4)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>/SKN/E_SW_STATE_ICON</t>
+          <t>MODBE</t>
         </is>
       </c>
     </row>
@@ -841,22 +829,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LOCNT</t>
+          <t>NO_DATE_RESTRICTION</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Number of failed logon attempts</t>
+          <t>NO_DATE_RESTRICTION</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>INT1(3)</t>
+          <t>CHAR(1)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>XULOCNT</t>
+          <t>NO_DATE_RESTRICTION</t>
         </is>
       </c>
     </row>
@@ -868,22 +856,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LTIME</t>
+          <t>PWDLGNDATE</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Last Logon Time</t>
+          <t>PWDLGNDATE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>TIMS(6)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>XULTIME</t>
+          <t>PWDLGNDATE</t>
         </is>
       </c>
     </row>
@@ -895,22 +883,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MODBE</t>
+          <t>PWDLOCKDATE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Last Changed By</t>
+          <t>PWDLOCKDATE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>XUMODIFIER</t>
+          <t>PWDLOCKDATE</t>
         </is>
       </c>
     </row>
@@ -922,22 +910,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MODDATE</t>
+          <t>PWDSETDATE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Modification date</t>
+          <t>PWDSETDATE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DATS(8)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>XUMODDATE</t>
+          <t>PWDSETDATE</t>
         </is>
       </c>
     </row>
@@ -949,22 +937,22 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>MODIFIER</t>
+          <t>STATE_COLOR</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Last Changed By</t>
+          <t>STATE_COLOR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CHAR(12)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>XUMODIFIER</t>
+          <t>STATE_COLOR</t>
         </is>
       </c>
     </row>
@@ -976,22 +964,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MODTIME</t>
+          <t>TRDAT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Modification time</t>
+          <t>TRDAT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TIMS(6)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>XUMODTIME</t>
+          <t>TRDAT</t>
         </is>
       </c>
     </row>
@@ -1003,22 +991,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NAME_FIRST</t>
+          <t>UFLAG</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>First name</t>
+          <t>UFLAG</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CHAR(40)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AD_NAMEFIR</t>
+          <t>UFLAG</t>
         </is>
       </c>
     </row>
@@ -1030,22 +1018,22 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NAME_LAST</t>
+          <t>USTYP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Last name</t>
+          <t>USTYP</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CHAR(40)</t>
+          <t>CHAR(50)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AD_NAMELAS</t>
+          <t>USTYP</t>
         </is>
       </c>
     </row>
@@ -1057,265 +1045,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NAME_TEXT</t>
+          <t>VALID_USERS_ONLY</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Full Name of Person</t>
+          <t>VALID_USERS_ONLY</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CHAR(80)</t>
+          <t>CHAR(1)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AD_NAMTEXT</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>PWDLGNDATE</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Date of Last Password Logon</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>DATS(8)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>XULPDAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>STATE_COLOR</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>SW: State Color</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>CHAR(1)</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>/SKN/E_SW_STATE_COLOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>STATE_DESC</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>SW: Message</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>CHAR(255)</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>/SKN/E_SW_TEXT</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>STATE_ICON</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>SW: State Icon</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>CHAR(4)</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>/SKN/E_SW_STATE_ICON</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>TRDAT</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Last Logon Date</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>DATS(8)</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>XULDATE</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>TZONE</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Time Zone</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>CHAR(6)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>TZNZONE</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>UFLAG</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>User Lock Status</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>INT1(3)</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>XUUFLAG</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>USTYP</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>User Type</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>CHAR(1)</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>XUUSTYP</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>/SKN/S_SW_01_20_USER_STATE</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>VERSN</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>User master record version</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>CHAR(3)</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>XUVERSION</t>
+          <t>VALID_USERS_ONLY</t>
         </is>
       </c>
     </row>

</xml_diff>